<commit_message>
water tank commode added
</commit_message>
<xml_diff>
--- a/2083_2084/estimate/budget maag estimate/Ward swasthya water tank/size water tank.xlsx
+++ b/2083_2084/estimate/budget maag estimate/Ward swasthya water tank/size water tank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\2083_2084\estimate\budget maag estimate\Ward swasthya water tank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE3AD85-F013-4341-8D2F-255338A121BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C05AD076-0EDD-4CAD-8569-BFB0884326B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'include dhara marmat'!$A$1:$K$173</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'water tank estimate'!$A$1:$K$315</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'water tank estimate'!$A$1:$K$320</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'include dhara marmat'!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'water tank estimate'!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">WCR!$1:$11</definedName>
@@ -217,7 +217,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="227">
   <si>
     <t>S.N.</t>
   </si>
@@ -987,6 +987,12 @@
   </si>
   <si>
     <t>-at outer face of staircase area</t>
+  </si>
+  <si>
+    <t>White glazed porcelain clay EWC floor mounted commode without cistern all complete set.</t>
+  </si>
+  <si>
+    <t>-for toilet at swasthya</t>
   </si>
 </sst>
 </file>
@@ -9778,7 +9784,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD07E67D-5D7A-4E99-87D9-10A521F06797}">
-  <dimension ref="A1:S316"/>
+  <dimension ref="A1:S321"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="4.42578125" style="69" customWidth="1"/>
@@ -16267,217 +16273,209 @@
       <c r="J303" s="80"/>
       <c r="K303" s="81"/>
     </row>
-    <row r="304" spans="1:11" ht="47.25" customHeight="1">
+    <row r="304" spans="1:11" ht="47.25">
       <c r="A304" s="77">
         <v>29</v>
       </c>
-      <c r="B304" s="93" t="s">
-        <v>187</v>
-      </c>
-      <c r="C304" s="83">
-        <v>1</v>
-      </c>
+      <c r="B304" s="120" t="s">
+        <v>225</v>
+      </c>
+      <c r="C304" s="83"/>
       <c r="D304" s="80"/>
       <c r="E304" s="80"/>
       <c r="F304" s="80"/>
-      <c r="G304" s="80">
-        <v>1</v>
-      </c>
-      <c r="H304" s="80" t="s">
-        <v>128</v>
-      </c>
-      <c r="I304" s="84">
-        <v>25000</v>
-      </c>
-      <c r="J304" s="84">
-        <f>G304*I304</f>
-        <v>25000</v>
-      </c>
+      <c r="G304" s="80"/>
+      <c r="H304" s="80"/>
+      <c r="I304" s="80"/>
+      <c r="J304" s="80"/>
       <c r="K304" s="81"/>
     </row>
     <row r="305" spans="1:11">
       <c r="A305" s="77"/>
-      <c r="B305" s="99"/>
-      <c r="C305" s="83"/>
+      <c r="B305" s="94" t="s">
+        <v>226</v>
+      </c>
+      <c r="C305" s="83">
+        <v>1</v>
+      </c>
       <c r="D305" s="80"/>
       <c r="E305" s="80"/>
-      <c r="F305" s="84"/>
-      <c r="G305" s="80"/>
+      <c r="F305" s="80"/>
+      <c r="G305" s="84">
+        <f t="shared" ref="G305" si="43">PRODUCT(C305:F305)</f>
+        <v>1</v>
+      </c>
       <c r="H305" s="80"/>
-      <c r="I305" s="84"/>
-      <c r="J305" s="84"/>
+      <c r="I305" s="80"/>
+      <c r="J305" s="80"/>
       <c r="K305" s="81"/>
     </row>
-    <row r="306" spans="1:11" ht="33" customHeight="1">
-      <c r="A306" s="77">
-        <v>30</v>
-      </c>
-      <c r="B306" s="93" t="s">
-        <v>75</v>
-      </c>
-      <c r="C306" s="83">
-        <v>1</v>
-      </c>
+    <row r="306" spans="1:11">
+      <c r="A306" s="77"/>
+      <c r="B306" s="92"/>
+      <c r="C306" s="83"/>
       <c r="D306" s="80"/>
       <c r="E306" s="80"/>
       <c r="F306" s="80"/>
       <c r="G306" s="80">
+        <f>SUM(G305:G305)</f>
         <v>1</v>
       </c>
       <c r="H306" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="I306" s="80">
+        <v>8656</v>
+      </c>
+      <c r="J306" s="80">
+        <f>G306*I306</f>
+        <v>8656</v>
+      </c>
+      <c r="K306" s="81"/>
+    </row>
+    <row r="307" spans="1:11">
+      <c r="A307" s="77"/>
+      <c r="B307" s="94" t="s">
+        <v>146</v>
+      </c>
+      <c r="C307" s="83"/>
+      <c r="D307" s="80"/>
+      <c r="E307" s="80"/>
+      <c r="F307" s="80"/>
+      <c r="G307" s="80"/>
+      <c r="H307" s="80"/>
+      <c r="I307" s="80"/>
+      <c r="J307" s="80">
+        <f>0.13*J306</f>
+        <v>1125.28</v>
+      </c>
+      <c r="K307" s="81"/>
+    </row>
+    <row r="308" spans="1:11">
+      <c r="A308" s="77"/>
+      <c r="B308" s="92"/>
+      <c r="C308" s="83"/>
+      <c r="D308" s="80"/>
+      <c r="E308" s="80"/>
+      <c r="F308" s="80"/>
+      <c r="G308" s="80"/>
+      <c r="H308" s="80"/>
+      <c r="I308" s="80"/>
+      <c r="J308" s="80"/>
+      <c r="K308" s="81"/>
+    </row>
+    <row r="309" spans="1:11" ht="47.25" customHeight="1">
+      <c r="A309" s="77">
+        <v>30</v>
+      </c>
+      <c r="B309" s="93" t="s">
+        <v>187</v>
+      </c>
+      <c r="C309" s="83">
+        <v>1</v>
+      </c>
+      <c r="D309" s="80"/>
+      <c r="E309" s="80"/>
+      <c r="F309" s="80"/>
+      <c r="G309" s="80">
+        <v>1</v>
+      </c>
+      <c r="H309" s="80" t="s">
+        <v>128</v>
+      </c>
+      <c r="I309" s="84">
+        <v>25000</v>
+      </c>
+      <c r="J309" s="84">
+        <f>G309*I309</f>
+        <v>25000</v>
+      </c>
+      <c r="K309" s="81"/>
+    </row>
+    <row r="310" spans="1:11">
+      <c r="A310" s="77"/>
+      <c r="B310" s="99"/>
+      <c r="C310" s="83"/>
+      <c r="D310" s="80"/>
+      <c r="E310" s="80"/>
+      <c r="F310" s="84"/>
+      <c r="G310" s="80"/>
+      <c r="H310" s="80"/>
+      <c r="I310" s="84"/>
+      <c r="J310" s="84"/>
+      <c r="K310" s="81"/>
+    </row>
+    <row r="311" spans="1:11" ht="33" customHeight="1">
+      <c r="A311" s="77">
+        <v>31</v>
+      </c>
+      <c r="B311" s="93" t="s">
+        <v>75</v>
+      </c>
+      <c r="C311" s="83">
+        <v>1</v>
+      </c>
+      <c r="D311" s="80"/>
+      <c r="E311" s="80"/>
+      <c r="F311" s="80"/>
+      <c r="G311" s="80">
+        <v>1</v>
+      </c>
+      <c r="H311" s="80" t="s">
         <v>33</v>
       </c>
-      <c r="I306" s="84">
+      <c r="I311" s="84">
         <v>500</v>
       </c>
-      <c r="J306" s="84">
-        <f>G306*I306</f>
+      <c r="J311" s="84">
+        <f>G311*I311</f>
         <v>500</v>
       </c>
-      <c r="K306" s="81"/>
-    </row>
-    <row r="307" spans="1:11">
-      <c r="A307" s="100"/>
-      <c r="B307" s="101"/>
-      <c r="C307" s="80"/>
-      <c r="D307" s="84"/>
-      <c r="E307" s="84"/>
-      <c r="F307" s="84"/>
-      <c r="G307" s="84"/>
-      <c r="H307" s="80"/>
-      <c r="I307" s="84"/>
-      <c r="J307" s="102">
-        <f>SUM(J12:J306)</f>
-        <v>1189146.8674031552</v>
-      </c>
-      <c r="K307" s="103"/>
-    </row>
-    <row r="308" spans="1:11">
-      <c r="A308" s="104"/>
-      <c r="B308" s="105"/>
-      <c r="C308" s="65"/>
-      <c r="D308" s="65"/>
-      <c r="E308" s="65"/>
-      <c r="F308" s="65"/>
-      <c r="G308" s="65"/>
-      <c r="H308" s="65"/>
-      <c r="I308" s="65"/>
-      <c r="J308" s="106"/>
-      <c r="K308" s="107"/>
-    </row>
-    <row r="309" spans="1:11">
-      <c r="A309" s="104"/>
-      <c r="B309" s="75" t="s">
-        <v>12</v>
-      </c>
-      <c r="C309" s="149" t="s">
-        <v>66</v>
-      </c>
-      <c r="D309" s="149"/>
-      <c r="E309" s="75" t="s">
-        <v>67</v>
-      </c>
-      <c r="F309" s="108"/>
-      <c r="G309" s="109"/>
-      <c r="H309" s="108"/>
-      <c r="I309" s="109"/>
-      <c r="J309" s="108"/>
-      <c r="K309" s="108"/>
-    </row>
-    <row r="310" spans="1:11">
-      <c r="A310" s="104"/>
-      <c r="B310" s="79" t="s">
-        <v>13</v>
-      </c>
-      <c r="C310" s="150">
-        <f>+J307</f>
-        <v>1189146.8674031552</v>
-      </c>
-      <c r="D310" s="150"/>
-      <c r="E310" s="110"/>
-      <c r="F310" s="108"/>
-      <c r="G310" s="111"/>
-      <c r="H310" s="108"/>
-      <c r="I310" s="109"/>
-      <c r="J310" s="108"/>
-      <c r="K310" s="108"/>
-    </row>
-    <row r="311" spans="1:11">
-      <c r="A311" s="104"/>
-      <c r="B311" s="79" t="s">
-        <v>14</v>
-      </c>
-      <c r="C311" s="150">
-        <v>1050000</v>
-      </c>
-      <c r="D311" s="150"/>
-      <c r="E311" s="112">
-        <v>100</v>
-      </c>
-      <c r="F311" s="108"/>
-      <c r="G311" s="111"/>
-      <c r="H311" s="108"/>
-      <c r="I311" s="109"/>
-      <c r="J311" s="108"/>
-      <c r="K311" s="108"/>
+      <c r="K311" s="81"/>
     </row>
     <row r="312" spans="1:11">
-      <c r="A312" s="104"/>
-      <c r="B312" s="79" t="s">
-        <v>19</v>
-      </c>
-      <c r="C312" s="150">
-        <f>0.95*C311</f>
-        <v>997500</v>
-      </c>
-      <c r="D312" s="150"/>
-      <c r="E312" s="113">
-        <f>C312/C310*100</f>
-        <v>83.883667135105739</v>
-      </c>
-      <c r="F312" s="108"/>
-      <c r="G312" s="111"/>
-      <c r="H312" s="108"/>
-      <c r="I312" s="109"/>
-      <c r="J312" s="108"/>
-      <c r="K312" s="108"/>
+      <c r="A312" s="100"/>
+      <c r="B312" s="101"/>
+      <c r="C312" s="80"/>
+      <c r="D312" s="84"/>
+      <c r="E312" s="84"/>
+      <c r="F312" s="84"/>
+      <c r="G312" s="84"/>
+      <c r="H312" s="80"/>
+      <c r="I312" s="84"/>
+      <c r="J312" s="102">
+        <f>SUM(J12:J311)</f>
+        <v>1198928.1474031552</v>
+      </c>
+      <c r="K312" s="103"/>
     </row>
     <row r="313" spans="1:11">
       <c r="A313" s="104"/>
-      <c r="B313" s="79" t="s">
-        <v>15</v>
-      </c>
-      <c r="C313" s="150">
-        <f>C310-C312</f>
-        <v>191646.86740315519</v>
-      </c>
-      <c r="D313" s="150"/>
-      <c r="E313" s="113">
-        <f>C313/C311*100</f>
-        <v>18.252082609824306</v>
-      </c>
-      <c r="F313" s="108"/>
-      <c r="G313" s="111"/>
-      <c r="H313" s="108"/>
-      <c r="I313" s="109"/>
-      <c r="J313" s="108"/>
-      <c r="K313" s="108"/>
+      <c r="B313" s="105"/>
+      <c r="C313" s="65"/>
+      <c r="D313" s="65"/>
+      <c r="E313" s="65"/>
+      <c r="F313" s="65"/>
+      <c r="G313" s="65"/>
+      <c r="H313" s="65"/>
+      <c r="I313" s="65"/>
+      <c r="J313" s="106"/>
+      <c r="K313" s="107"/>
     </row>
     <row r="314" spans="1:11">
       <c r="A314" s="104"/>
-      <c r="B314" s="79" t="s">
-        <v>20</v>
-      </c>
-      <c r="C314" s="150">
-        <f>E314*C311/100</f>
-        <v>21000</v>
-      </c>
-      <c r="D314" s="150"/>
-      <c r="E314" s="113">
-        <v>2</v>
+      <c r="B314" s="75" t="s">
+        <v>12</v>
+      </c>
+      <c r="C314" s="149" t="s">
+        <v>66</v>
+      </c>
+      <c r="D314" s="149"/>
+      <c r="E314" s="75" t="s">
+        <v>67</v>
       </c>
       <c r="F314" s="108"/>
-      <c r="G314" s="111"/>
+      <c r="G314" s="109"/>
       <c r="H314" s="108"/>
       <c r="I314" s="109"/>
       <c r="J314" s="108"/>
@@ -16486,25 +16484,124 @@
     <row r="315" spans="1:11">
       <c r="A315" s="104"/>
       <c r="B315" s="79" t="s">
-        <v>21</v>
-      </c>
-      <c r="C315" s="148">
-        <f>E315*C311/100</f>
-        <v>31500</v>
-      </c>
-      <c r="D315" s="148"/>
-      <c r="E315" s="113">
-        <v>3</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C315" s="150">
+        <f>+J312</f>
+        <v>1198928.1474031552</v>
+      </c>
+      <c r="D315" s="150"/>
+      <c r="E315" s="110"/>
       <c r="F315" s="108"/>
-      <c r="G315" s="114"/>
+      <c r="G315" s="111"/>
       <c r="H315" s="108"/>
       <c r="I315" s="109"/>
       <c r="J315" s="108"/>
       <c r="K315" s="108"/>
     </row>
     <row r="316" spans="1:11">
-      <c r="F316" s="37"/>
+      <c r="A316" s="104"/>
+      <c r="B316" s="79" t="s">
+        <v>14</v>
+      </c>
+      <c r="C316" s="150">
+        <v>1050000</v>
+      </c>
+      <c r="D316" s="150"/>
+      <c r="E316" s="112">
+        <v>100</v>
+      </c>
+      <c r="F316" s="108"/>
+      <c r="G316" s="111"/>
+      <c r="H316" s="108"/>
+      <c r="I316" s="109"/>
+      <c r="J316" s="108"/>
+      <c r="K316" s="108"/>
+    </row>
+    <row r="317" spans="1:11">
+      <c r="A317" s="104"/>
+      <c r="B317" s="79" t="s">
+        <v>19</v>
+      </c>
+      <c r="C317" s="150">
+        <f>0.95*C316</f>
+        <v>997500</v>
+      </c>
+      <c r="D317" s="150"/>
+      <c r="E317" s="113">
+        <f>C317/C315*100</f>
+        <v>83.199314501086405</v>
+      </c>
+      <c r="F317" s="108"/>
+      <c r="G317" s="111"/>
+      <c r="H317" s="108"/>
+      <c r="I317" s="109"/>
+      <c r="J317" s="108"/>
+      <c r="K317" s="108"/>
+    </row>
+    <row r="318" spans="1:11">
+      <c r="A318" s="104"/>
+      <c r="B318" s="79" t="s">
+        <v>15</v>
+      </c>
+      <c r="C318" s="150">
+        <f>C315-C317</f>
+        <v>201428.14740315522</v>
+      </c>
+      <c r="D318" s="150"/>
+      <c r="E318" s="113">
+        <f>C318/C316*100</f>
+        <v>19.183633086014783</v>
+      </c>
+      <c r="F318" s="108"/>
+      <c r="G318" s="111"/>
+      <c r="H318" s="108"/>
+      <c r="I318" s="109"/>
+      <c r="J318" s="108"/>
+      <c r="K318" s="108"/>
+    </row>
+    <row r="319" spans="1:11">
+      <c r="A319" s="104"/>
+      <c r="B319" s="79" t="s">
+        <v>20</v>
+      </c>
+      <c r="C319" s="150">
+        <f>E319*C316/100</f>
+        <v>21000</v>
+      </c>
+      <c r="D319" s="150"/>
+      <c r="E319" s="113">
+        <v>2</v>
+      </c>
+      <c r="F319" s="108"/>
+      <c r="G319" s="111"/>
+      <c r="H319" s="108"/>
+      <c r="I319" s="109"/>
+      <c r="J319" s="108"/>
+      <c r="K319" s="108"/>
+    </row>
+    <row r="320" spans="1:11">
+      <c r="A320" s="104"/>
+      <c r="B320" s="79" t="s">
+        <v>21</v>
+      </c>
+      <c r="C320" s="148">
+        <f>E320*C316/100</f>
+        <v>31500</v>
+      </c>
+      <c r="D320" s="148"/>
+      <c r="E320" s="113">
+        <v>3</v>
+      </c>
+      <c r="F320" s="108"/>
+      <c r="G320" s="114"/>
+      <c r="H320" s="108"/>
+      <c r="I320" s="109"/>
+      <c r="J320" s="108"/>
+      <c r="K320" s="108"/>
+    </row>
+    <row r="321" spans="6:6">
+      <c r="F321" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -16515,13 +16612,13 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="J5:K5"/>
+    <mergeCell ref="C320:D320"/>
+    <mergeCell ref="C314:D314"/>
     <mergeCell ref="C315:D315"/>
-    <mergeCell ref="C309:D309"/>
-    <mergeCell ref="C310:D310"/>
-    <mergeCell ref="C311:D311"/>
-    <mergeCell ref="C312:D312"/>
-    <mergeCell ref="C313:D313"/>
-    <mergeCell ref="C314:D314"/>
+    <mergeCell ref="C316:D316"/>
+    <mergeCell ref="C317:D317"/>
+    <mergeCell ref="C318:D318"/>
+    <mergeCell ref="C319:D319"/>
   </mergeCells>
   <phoneticPr fontId="84" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>